<commit_message>
Visor compartido: secuencia y etiquetas configurables desde la hoja RED, tipos de fuente ampliados
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/red-sintomas-kennedy.xlsx
+++ b/datos/red-sintomas-kennedy.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5768" uniqueCount="1966">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5772" uniqueCount="1970">
   <si>
     <t>RED DE SÍNTOMAS Y EFECTOS DE KENNEDY — ENFOQUES: ECONOMÍA, INNOVACIÓN, REDES (Y METABOLISMO)</t>
   </si>
@@ -5822,6 +5822,18 @@
   </si>
   <si>
     <t>capa_clave</t>
+  </si>
+  <si>
+    <t>secuencia</t>
+  </si>
+  <si>
+    <t>si</t>
+  </si>
+  <si>
+    <t>saludo</t>
+  </si>
+  <si>
+    <t>la red de síntomas y efectos de Kennedy</t>
   </si>
   <si>
     <t>fuentes</t>
@@ -27247,7 +27259,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -27364,6 +27376,22 @@
       </c>
       <c r="B14" t="s">
         <v>1952</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>1953</v>
+      </c>
+      <c r="B15" t="s">
+        <v>1954</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>1955</v>
+      </c>
+      <c r="B16" t="s">
+        <v>1956</v>
       </c>
     </row>
   </sheetData>
@@ -27384,18 +27412,18 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>1953</v>
+        <v>1957</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>1954</v>
+        <v>1958</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>1955</v>
+        <v>1959</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>1956</v>
+        <v>1960</v>
       </c>
       <c r="B2">
         <f>SUMPRODUCT((COUNTIF(NODOS!A2:A500,NODOS!A2:A500)&gt;1)*(NODOS!A2:A500&lt;&gt;""))</f>
@@ -27406,7 +27434,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>1957</v>
+        <v>1961</v>
       </c>
       <c r="B3">
         <f>SUMPRODUCT((NODOS!A2:A500&lt;&gt;"")*(COUNTIF(CAPAS!B2:B30,NODOS!C2:C500)=0))</f>
@@ -27417,7 +27445,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>1958</v>
+        <v>1962</v>
       </c>
       <c r="B4">
         <f>SUMPRODUCT((ARISTAS!A2:A500&lt;&gt;"")*(COUNTIF(NODOS!A2:A500,ARISTAS!B2:B500)=0))</f>
@@ -27428,7 +27456,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>1959</v>
+        <v>1963</v>
       </c>
       <c r="B5">
         <f>SUMPRODUCT((ARISTAS!A2:A500&lt;&gt;"")*(COUNTIF(NODOS!A2:A500,ARISTAS!C2:C500)=0))</f>
@@ -27439,7 +27467,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>1960</v>
+        <v>1964</v>
       </c>
       <c r="B6">
         <f>SUMPRODUCT((ARISTAS!A2:A500&lt;&gt;"")*(COUNTIF(INTERACCIONES!B2:B30,ARISTAS!D2:D500)=0))</f>
@@ -27450,7 +27478,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>1961</v>
+        <v>1965</v>
       </c>
       <c r="B7">
         <f>SUMPRODUCT((ARISTAS!A2:A500&lt;&gt;"")*(ARISTAS!B2:B500=ARISTAS!C2:C500))</f>
@@ -27461,7 +27489,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>1962</v>
+        <v>1966</v>
       </c>
       <c r="B8">
         <f>SUMPRODUCT((NODOS!A2:A500&lt;&gt;"")*(COUNTIF(ARISTAS!B2:B500,NODOS!A2:A500)+COUNTIF(ARISTAS!C2:C500,NODOS!A2:A500)=0))</f>
@@ -27472,7 +27500,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>1963</v>
+        <v>1967</v>
       </c>
       <c r="B9" t="s">
         <v>1</v>
@@ -27483,7 +27511,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>1964</v>
+        <v>1968</v>
       </c>
       <c r="B10">
         <f>COUNTA(NODOS!A2:A500)</f>
@@ -27491,7 +27519,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>1965</v>
+        <v>1969</v>
       </c>
       <c r="B11">
         <f>COUNTA(ARISTAS!A2:A500)</f>

</xml_diff>